<commit_message>
Fix DECISION scope bug · hoist PRIORITY_MATRIX + vocab loader to top of _split_and_send
Previous commit had UnboundLocalError · PRIORITY_MATRIX defined AFTER
row iteration loop that referenced it. Hoisted config loaders + resolver
to top of _split_and_send so both Portfolio and History sheet builders
can reference. Verified both sheets both markets now have DECISION +
Urgency + Reason + Action + Review columns.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/telegram/aegis_history_usa.xlsx
+++ b/reports/telegram/aegis_history_usa.xlsx
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY1"/>
+  <dimension ref="A1:BD1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -740,7 +740,7 @@
     <col width="12" customWidth="1" min="24" max="24"/>
     <col width="6" customWidth="1" min="25" max="25"/>
     <col width="13" customWidth="1" min="26" max="26"/>
-    <col width="18" customWidth="1" min="51" max="51"/>
+    <col width="18" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -997,6 +997,31 @@
       <c r="AY1" s="9" t="inlineStr">
         <is>
           <t>Inv Verdict</t>
+        </is>
+      </c>
+      <c r="AZ1" s="9" t="inlineStr">
+        <is>
+          <t>🎯 DECISION</t>
+        </is>
+      </c>
+      <c r="BA1" s="9" t="inlineStr">
+        <is>
+          <t>Urgency</t>
+        </is>
+      </c>
+      <c r="BB1" s="9" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+      <c r="BC1" s="9" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="BD1" s="9" t="inlineStr">
+        <is>
+          <t>Review</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Second chr(64+c) fixed at line 834 · Portfolio column widths · Execution Layer XLSX finally uncorrupted
Two chr(64+c) references existed · earlier fix only caught line 601 (source
sheet widths) · this fix catches line 834 (Portfolio sheet widths). Both
now use get_column_letter · handles A..Z, AA..AZ correctly.

Verified both markets both sheets have Price Trigger + Next Review +
Execution Window columns. XLSX files valid.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/telegram/aegis_history_usa.xlsx
+++ b/reports/telegram/aegis_history_usa.xlsx
@@ -1,3 +1,173 @@
+
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AEGIS USA History" sheetId="2" state="visible" r:id="rId2"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="+0.00%;-0.00%;0.00%"/>
+  </numFmts>
+  <fonts count="5">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
+  </fonts>
+  <fills count="4">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+        <bgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
@@ -280,4 +450,636 @@
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
+</file>
+
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AB7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="40" customWidth="1" min="26" max="26"/>
+    <col width="40" customWidth="1" min="27" max="27"/>
+    <col width="30" customWidth="1" min="28" max="28"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>AEGIS USA PORTFOLIO · as of today</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Realized P&amp;L (closed)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>0 closed</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Best position</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> +0.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Unrealized P&amp;L (open)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>0 open</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Worst position</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> +0.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>COMBINED PORTFOLIO</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>0 positions</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Win rate</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>0.0% (0W / 0L / 0 flat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>🎯 DECISION</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Price Trigger</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Next Review</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Execution Window</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Runner</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Cap</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Entry Date</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>Exit Date</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>Urgency</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="P7" s="8" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="Q7" s="8" t="inlineStr">
+        <is>
+          <t>Inv Quality</t>
+        </is>
+      </c>
+      <c r="R7" s="8" t="inlineStr">
+        <is>
+          <t>Investability</t>
+        </is>
+      </c>
+      <c r="S7" s="8" t="inlineStr">
+        <is>
+          <t>Entry</t>
+        </is>
+      </c>
+      <c r="T7" s="8" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="U7" s="8" t="inlineStr">
+        <is>
+          <t>Exit Price</t>
+        </is>
+      </c>
+      <c r="V7" s="8" t="inlineStr">
+        <is>
+          <t>P&amp;L %</t>
+        </is>
+      </c>
+      <c r="W7" s="8" t="inlineStr">
+        <is>
+          <t>Stop Loss</t>
+        </is>
+      </c>
+      <c r="X7" s="8" t="inlineStr">
+        <is>
+          <t>Target 1</t>
+        </is>
+      </c>
+      <c r="Y7" s="8" t="inlineStr">
+        <is>
+          <t>Target 2</t>
+        </is>
+      </c>
+      <c r="Z7" s="8" t="inlineStr">
+        <is>
+          <t>Action Note</t>
+        </is>
+      </c>
+      <c r="AA7" s="8" t="inlineStr">
+        <is>
+          <t>Alerts</t>
+        </is>
+      </c>
+      <c r="AB7" s="8" t="inlineStr">
+        <is>
+          <t>Exit Reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:BG1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="50" customWidth="1" min="19" max="19"/>
+    <col width="60" customWidth="1" min="20" max="20"/>
+    <col width="44" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="6" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="10" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
+    <col width="14" customWidth="1" min="30" max="30"/>
+    <col width="12" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="32" max="32"/>
+    <col width="13" customWidth="1" min="33" max="33"/>
+    <col width="11" customWidth="1" min="34" max="34"/>
+    <col width="9" customWidth="1" min="35" max="35"/>
+    <col width="11" customWidth="1" min="36" max="36"/>
+    <col width="8" customWidth="1" min="37" max="37"/>
+    <col width="11" customWidth="1" min="38" max="38"/>
+    <col width="8" customWidth="1" min="39" max="39"/>
+    <col width="11" customWidth="1" min="40" max="40"/>
+    <col width="13" customWidth="1" min="41" max="41"/>
+    <col width="15" customWidth="1" min="42" max="42"/>
+    <col width="12" customWidth="1" min="43" max="43"/>
+    <col width="11" customWidth="1" min="44" max="44"/>
+    <col width="32" customWidth="1" min="45" max="45"/>
+    <col width="20" customWidth="1" min="46" max="46"/>
+    <col width="18" customWidth="1" min="47" max="47"/>
+    <col width="18" customWidth="1" min="59" max="59"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Position ID</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Run_Type</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>Exit Reason</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>Exit P&amp;L %</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="K1" s="9" t="inlineStr">
+        <is>
+          <t>Prior Rank</t>
+        </is>
+      </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
+          <t>Rank Δ</t>
+        </is>
+      </c>
+      <c r="M1" s="9" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="N1" s="9" t="inlineStr">
+        <is>
+          <t>Risk Meter</t>
+        </is>
+      </c>
+      <c r="O1" s="9" t="inlineStr">
+        <is>
+          <t>Adj Conf</t>
+        </is>
+      </c>
+      <c r="P1" s="9" t="inlineStr">
+        <is>
+          <t>Ctx Drag</t>
+        </is>
+      </c>
+      <c r="Q1" s="9" t="inlineStr">
+        <is>
+          <t>Ctx Reason</t>
+        </is>
+      </c>
+      <c r="R1" s="9" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="S1" s="9" t="inlineStr">
+        <is>
+          <t>Alerts</t>
+        </is>
+      </c>
+      <c r="T1" s="9" t="inlineStr">
+        <is>
+          <t>Confidence %</t>
+        </is>
+      </c>
+      <c r="U1" s="9" t="inlineStr">
+        <is>
+          <t>Conf Type</t>
+        </is>
+      </c>
+      <c r="V1" s="9" t="inlineStr">
+        <is>
+          <t>Model Score</t>
+        </is>
+      </c>
+      <c r="W1" s="9" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="X1" s="9" t="inlineStr">
+        <is>
+          <t>Trading Days</t>
+        </is>
+      </c>
+      <c r="Y1" s="9" t="inlineStr">
+        <is>
+          <t>Horizon (d)</t>
+        </is>
+      </c>
+      <c r="Z1" s="9" t="inlineStr">
+        <is>
+          <t>Days Left</t>
+        </is>
+      </c>
+      <c r="AA1" s="9" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="AB1" s="9" t="inlineStr">
+        <is>
+          <t>Current Price</t>
+        </is>
+      </c>
+      <c r="AC1" s="9" t="inlineStr">
+        <is>
+          <t>Entry Price</t>
+        </is>
+      </c>
+      <c r="AD1" s="9" t="inlineStr">
+        <is>
+          <t>Buy Zone Low</t>
+        </is>
+      </c>
+      <c r="AE1" s="9" t="inlineStr">
+        <is>
+          <t>Buy Zone High</t>
+        </is>
+      </c>
+      <c r="AF1" s="9" t="inlineStr">
+        <is>
+          <t>Stop Loss</t>
+        </is>
+      </c>
+      <c r="AG1" s="9" t="inlineStr">
+        <is>
+          <t>Risk %</t>
+        </is>
+      </c>
+      <c r="AH1" s="9" t="inlineStr">
+        <is>
+          <t>Target 1</t>
+        </is>
+      </c>
+      <c r="AI1" s="9" t="inlineStr">
+        <is>
+          <t>T1 %</t>
+        </is>
+      </c>
+      <c r="AJ1" s="9" t="inlineStr">
+        <is>
+          <t>Target 2</t>
+        </is>
+      </c>
+      <c r="AK1" s="9" t="inlineStr">
+        <is>
+          <t>T2 %</t>
+        </is>
+      </c>
+      <c r="AL1" s="9" t="inlineStr">
+        <is>
+          <t>Prev Close</t>
+        </is>
+      </c>
+      <c r="AM1" s="9" t="inlineStr">
+        <is>
+          <t>Today Move %</t>
+        </is>
+      </c>
+      <c r="AN1" s="9" t="inlineStr">
+        <is>
+          <t>Current Perf %</t>
+        </is>
+      </c>
+      <c r="AO1" s="9" t="inlineStr">
+        <is>
+          <t>Max Gain %</t>
+        </is>
+      </c>
+      <c r="AP1" s="9" t="inlineStr">
+        <is>
+          <t>Max DD %</t>
+        </is>
+      </c>
+      <c r="AQ1" s="9" t="inlineStr">
+        <is>
+          <t>Top Drivers</t>
+        </is>
+      </c>
+      <c r="AR1" s="9" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="AS1" s="9" t="inlineStr">
+        <is>
+          <t>Portfolio Weight %</t>
+        </is>
+      </c>
+      <c r="AT1" s="9" t="inlineStr">
+        <is>
+          <t>Expected Alpha %</t>
+        </is>
+      </c>
+      <c r="AU1" s="9" t="inlineStr">
+        <is>
+          <t>Last Updated (UTC)</t>
+        </is>
+      </c>
+      <c r="AV1" s="9" t="inlineStr">
+        <is>
+          <t>Cap Size</t>
+        </is>
+      </c>
+      <c r="AW1" s="9" t="inlineStr">
+        <is>
+          <t>Opp Age</t>
+        </is>
+      </c>
+      <c r="AX1" s="9" t="inlineStr">
+        <is>
+          <t>Investability</t>
+        </is>
+      </c>
+      <c r="AY1" s="9" t="inlineStr">
+        <is>
+          <t>Inv Verdict</t>
+        </is>
+      </c>
+      <c r="AZ1" s="9" t="inlineStr">
+        <is>
+          <t>🎯 DECISION</t>
+        </is>
+      </c>
+      <c r="BA1" s="9" t="inlineStr">
+        <is>
+          <t>Urgency</t>
+        </is>
+      </c>
+      <c r="BB1" s="9" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+      <c r="BC1" s="9" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="BD1" s="9" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="BE1" s="9" t="inlineStr">
+        <is>
+          <t>Price Trigger</t>
+        </is>
+      </c>
+      <c r="BF1" s="9" t="inlineStr">
+        <is>
+          <t>Next Review</t>
+        </is>
+      </c>
+      <c r="BG1" s="9" t="inlineStr">
+        <is>
+          <t>Execution Window</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Same-day EXIT -> ARTIFACT + CI mark-only-on-send-success + both markets sent
- Priority classifier: same-day EXIT (Entry Date == Exit Date) reclassified
  as J (ARTIFACT) not I (CLOSED) · fixes USA -78 percent artifact aggregate
- CI workflow: mark data/.published only when steps.send.outcome==success ·
  fixes silent-fail retry no-op after Guard 8 block

Both markets sent (India 211 rows · USA 37 rows). Guard 10 India GREEN.
USA shows 12 RecDrift warnings (post-wipe recommendation date shifts) ·
non-blocking · to be investigated.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/telegram/aegis_history_usa.xlsx
+++ b/reports/telegram/aegis_history_usa.xlsx
@@ -86,14 +86,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6DCE4"/>
-        <bgColor rgb="00D6DCE4"/>
+        <fgColor rgb="00E7E6E6"/>
+        <bgColor rgb="00E7E6E6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E7E6E6"/>
-        <bgColor rgb="00E7E6E6"/>
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -602,7 +602,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AEGIS USA PORTFOLIO · as of 2026-08-10</t>
+          <t>AEGIS USA PORTFOLIO · as of 2026-08-11</t>
         </is>
       </c>
     </row>
@@ -841,29 +841,17 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>🟢 HOLD</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>🟡 REVIEWING</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>Review @ 333.74</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>🟠 No execution · investigate + decide</t>
-        </is>
-      </c>
+          <t>⚪ ARTIFACT</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr"/>
+      <c r="E8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr"/>
       <c r="G8" s="9" t="inlineStr">
         <is>
           <t>R2</t>
@@ -899,22 +887,22 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>🟡 MEDIUM</t>
+          <t>⚪ CLOSED</t>
         </is>
       </c>
       <c r="O8" s="9" t="inlineStr">
         <is>
-          <t>Premature Exit?</t>
+          <t>Artifact</t>
         </is>
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>5 DAYS</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="R8" s="9" t="inlineStr">
@@ -965,12 +953,12 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr"/>
@@ -1016,12 +1004,12 @@
       </c>
       <c r="O9" s="9" t="inlineStr">
         <is>
-          <t>Clean Exit</t>
+          <t>Artifact</t>
         </is>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
@@ -1071,12 +1059,12 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr"/>
@@ -1122,12 +1110,12 @@
       </c>
       <c r="O10" s="9" t="inlineStr">
         <is>
-          <t>Clean Exit</t>
+          <t>Artifact</t>
         </is>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
@@ -1177,12 +1165,12 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr"/>
@@ -1228,12 +1216,12 @@
       </c>
       <c r="O11" s="9" t="inlineStr">
         <is>
-          <t>Clean Exit</t>
+          <t>Artifact</t>
         </is>
       </c>
       <c r="P11" s="9" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="Q11" s="9" t="inlineStr">
@@ -1283,12 +1271,12 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr"/>
@@ -1334,12 +1322,12 @@
       </c>
       <c r="O12" s="9" t="inlineStr">
         <is>
-          <t>Clean Exit</t>
+          <t>Artifact</t>
         </is>
       </c>
       <c r="P12" s="9" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="Q12" s="9" t="inlineStr">
@@ -1389,12 +1377,12 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr"/>
@@ -1440,12 +1428,12 @@
       </c>
       <c r="O13" s="9" t="inlineStr">
         <is>
-          <t>Clean Exit</t>
+          <t>Artifact</t>
         </is>
       </c>
       <c r="P13" s="9" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="Q13" s="9" t="inlineStr">
@@ -1499,12 +1487,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr"/>
@@ -1550,12 +1538,12 @@
       </c>
       <c r="O14" s="9" t="inlineStr">
         <is>
-          <t>Clean Exit</t>
+          <t>Artifact</t>
         </is>
       </c>
       <c r="P14" s="9" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="Q14" s="9" t="inlineStr">
@@ -1609,12 +1597,12 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr"/>
@@ -1660,12 +1648,12 @@
       </c>
       <c r="O15" s="9" t="inlineStr">
         <is>
-          <t>Clean Exit</t>
+          <t>Artifact</t>
         </is>
       </c>
       <c r="P15" s="9" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="Q15" s="9" t="inlineStr">
@@ -1719,12 +1707,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr"/>
@@ -1770,12 +1758,12 @@
       </c>
       <c r="O16" s="9" t="inlineStr">
         <is>
-          <t>Clean Exit</t>
+          <t>Artifact</t>
         </is>
       </c>
       <c r="P16" s="9" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="Q16" s="9" t="inlineStr">
@@ -1829,12 +1817,12 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr"/>
@@ -1880,12 +1868,12 @@
       </c>
       <c r="O17" s="9" t="inlineStr">
         <is>
-          <t>Clean Exit</t>
+          <t>Artifact</t>
         </is>
       </c>
       <c r="P17" s="9" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="Q17" s="9" t="inlineStr">
@@ -1939,12 +1927,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr"/>
@@ -1990,12 +1978,12 @@
       </c>
       <c r="O18" s="9" t="inlineStr">
         <is>
-          <t>Clean Exit</t>
+          <t>Artifact</t>
         </is>
       </c>
       <c r="P18" s="9" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="Q18" s="9" t="inlineStr">
@@ -2049,12 +2037,12 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr"/>
@@ -2100,12 +2088,12 @@
       </c>
       <c r="O19" s="9" t="inlineStr">
         <is>
-          <t>Clean Exit</t>
+          <t>Artifact</t>
         </is>
       </c>
       <c r="P19" s="9" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="Q19" s="9" t="inlineStr">
@@ -2159,12 +2147,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>⚪ CLOSED</t>
+          <t>⚪ ARTIFACT</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr"/>
@@ -2210,12 +2198,12 @@
       </c>
       <c r="O20" s="9" t="inlineStr">
         <is>
-          <t>Clean Exit</t>
+          <t>Artifact</t>
         </is>
       </c>
       <c r="P20" s="9" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="Q20" s="9" t="inlineStr">
@@ -2284,37 +2272,37 @@
       </c>
       <c r="E21" s="16" t="inlineStr">
         <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>✅ AGREE</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
           <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="F21" s="16" t="inlineStr">
-        <is>
-          <t>🟡 Normal window · 10:00-14:30 IST</t>
-        </is>
-      </c>
-      <c r="G21" s="16" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="H21" s="16" t="inlineStr">
-        <is>
-          <t>✅ AGREE</t>
-        </is>
-      </c>
-      <c r="I21" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J21" s="16" t="inlineStr">
-        <is>
-          <t>LargeCap (S&amp;P 500)</t>
-        </is>
-      </c>
-      <c r="K21" s="16" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L21" s="16" t="n"/>
@@ -2398,37 +2386,37 @@
       </c>
       <c r="E22" s="22" t="inlineStr">
         <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+      <c r="G22" s="22" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="H22" s="22" t="inlineStr">
+        <is>
+          <t>✅ AGREE</t>
+        </is>
+      </c>
+      <c r="I22" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J22" s="22" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="K22" s="22" t="inlineStr">
+        <is>
           <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="F22" s="22" t="inlineStr">
-        <is>
-          <t>🟡 Normal window · 10:00-14:30 IST</t>
-        </is>
-      </c>
-      <c r="G22" s="22" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="H22" s="22" t="inlineStr">
-        <is>
-          <t>✅ AGREE</t>
-        </is>
-      </c>
-      <c r="I22" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J22" s="22" t="inlineStr">
-        <is>
-          <t>LargeCap (S&amp;P 500)</t>
-        </is>
-      </c>
-      <c r="K22" s="22" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L22" s="22" t="n"/>
@@ -2512,37 +2500,37 @@
       </c>
       <c r="E23" s="16" t="inlineStr">
         <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+      <c r="G23" s="16" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>✅ AGREE</t>
+        </is>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="K23" s="16" t="inlineStr">
+        <is>
           <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>🟡 Normal window · 10:00-14:30 IST</t>
-        </is>
-      </c>
-      <c r="G23" s="16" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H23" s="16" t="inlineStr">
-        <is>
-          <t>✅ AGREE</t>
-        </is>
-      </c>
-      <c r="I23" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J23" s="16" t="inlineStr">
-        <is>
-          <t>LargeCap (S&amp;P 500)</t>
-        </is>
-      </c>
-      <c r="K23" s="16" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L23" s="16" t="n"/>
@@ -2626,37 +2614,37 @@
       </c>
       <c r="E24" s="16" t="inlineStr">
         <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+      <c r="G24" s="16" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H24" s="16" t="inlineStr">
+        <is>
+          <t>✅ AGREE</t>
+        </is>
+      </c>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J24" s="16" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="K24" s="16" t="inlineStr">
+        <is>
           <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="F24" s="16" t="inlineStr">
-        <is>
-          <t>🟡 Normal window · 10:00-14:30 IST</t>
-        </is>
-      </c>
-      <c r="G24" s="16" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H24" s="16" t="inlineStr">
-        <is>
-          <t>✅ AGREE</t>
-        </is>
-      </c>
-      <c r="I24" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J24" s="16" t="inlineStr">
-        <is>
-          <t>LargeCap (S&amp;P 500)</t>
-        </is>
-      </c>
-      <c r="K24" s="16" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L24" s="16" t="n"/>
@@ -2740,37 +2728,37 @@
       </c>
       <c r="E25" s="16" t="inlineStr">
         <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+      <c r="G25" s="16" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>✅ AGREE</t>
+        </is>
+      </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J25" s="16" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="K25" s="16" t="inlineStr">
+        <is>
           <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="F25" s="16" t="inlineStr">
-        <is>
-          <t>🟡 Normal window · 10:00-14:30 IST</t>
-        </is>
-      </c>
-      <c r="G25" s="16" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H25" s="16" t="inlineStr">
-        <is>
-          <t>✅ AGREE</t>
-        </is>
-      </c>
-      <c r="I25" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J25" s="16" t="inlineStr">
-        <is>
-          <t>LargeCap (S&amp;P 500)</t>
-        </is>
-      </c>
-      <c r="K25" s="16" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L25" s="16" t="n"/>
@@ -2858,37 +2846,37 @@
       </c>
       <c r="E26" s="16" t="inlineStr">
         <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+      <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H26" s="16" t="inlineStr">
+        <is>
+          <t>✅ AGREE</t>
+        </is>
+      </c>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J26" s="16" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="K26" s="16" t="inlineStr">
+        <is>
           <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="F26" s="16" t="inlineStr">
-        <is>
-          <t>🟡 Normal window · 10:00-14:30 IST</t>
-        </is>
-      </c>
-      <c r="G26" s="16" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H26" s="16" t="inlineStr">
-        <is>
-          <t>✅ AGREE</t>
-        </is>
-      </c>
-      <c r="I26" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J26" s="16" t="inlineStr">
-        <is>
-          <t>LargeCap (S&amp;P 500)</t>
-        </is>
-      </c>
-      <c r="K26" s="16" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L26" s="16" t="n"/>
@@ -2976,37 +2964,37 @@
       </c>
       <c r="E27" s="22" t="inlineStr">
         <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F27" s="22" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+      <c r="G27" s="22" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H27" s="22" t="inlineStr">
+        <is>
+          <t>✅ AGREE</t>
+        </is>
+      </c>
+      <c r="I27" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J27" s="22" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="K27" s="22" t="inlineStr">
+        <is>
           <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="F27" s="22" t="inlineStr">
-        <is>
-          <t>🟡 Normal window · 10:00-14:30 IST</t>
-        </is>
-      </c>
-      <c r="G27" s="22" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H27" s="22" t="inlineStr">
-        <is>
-          <t>✅ AGREE</t>
-        </is>
-      </c>
-      <c r="I27" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J27" s="22" t="inlineStr">
-        <is>
-          <t>LargeCap (S&amp;P 500)</t>
-        </is>
-      </c>
-      <c r="K27" s="22" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L27" s="22" t="n"/>
@@ -3094,37 +3082,37 @@
       </c>
       <c r="E28" s="22" t="inlineStr">
         <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F28" s="22" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+      <c r="G28" s="22" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H28" s="22" t="inlineStr">
+        <is>
+          <t>✅ AGREE</t>
+        </is>
+      </c>
+      <c r="I28" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J28" s="22" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="K28" s="22" t="inlineStr">
+        <is>
           <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="F28" s="22" t="inlineStr">
-        <is>
-          <t>🟡 Normal window · 10:00-14:30 IST</t>
-        </is>
-      </c>
-      <c r="G28" s="22" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H28" s="22" t="inlineStr">
-        <is>
-          <t>✅ AGREE</t>
-        </is>
-      </c>
-      <c r="I28" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J28" s="22" t="inlineStr">
-        <is>
-          <t>LargeCap (S&amp;P 500)</t>
-        </is>
-      </c>
-      <c r="K28" s="22" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L28" s="22" t="n"/>
@@ -3212,7 +3200,7 @@
       </c>
       <c r="E29" s="22" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F29" s="22" t="inlineStr">
@@ -3242,7 +3230,7 @@
       </c>
       <c r="K29" s="22" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="L29" s="22" t="n"/>
@@ -3332,37 +3320,37 @@
       </c>
       <c r="E30" s="22" t="inlineStr">
         <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F30" s="22" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+      <c r="G30" s="22" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H30" s="22" t="inlineStr">
+        <is>
+          <t>✅ AGREE</t>
+        </is>
+      </c>
+      <c r="I30" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J30" s="22" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="K30" s="22" t="inlineStr">
+        <is>
           <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="F30" s="22" t="inlineStr">
-        <is>
-          <t>🟡 Normal window · 10:00-14:30 IST</t>
-        </is>
-      </c>
-      <c r="G30" s="22" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H30" s="22" t="inlineStr">
-        <is>
-          <t>✅ AGREE</t>
-        </is>
-      </c>
-      <c r="I30" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J30" s="22" t="inlineStr">
-        <is>
-          <t>LargeCap (S&amp;P 500)</t>
-        </is>
-      </c>
-      <c r="K30" s="22" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L30" s="22" t="n"/>
@@ -3450,37 +3438,37 @@
       </c>
       <c r="E31" s="22" t="inlineStr">
         <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F31" s="22" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+      <c r="G31" s="22" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H31" s="22" t="inlineStr">
+        <is>
+          <t>✅ AGREE</t>
+        </is>
+      </c>
+      <c r="I31" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J31" s="22" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="K31" s="22" t="inlineStr">
+        <is>
           <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="F31" s="22" t="inlineStr">
-        <is>
-          <t>🟡 Normal window · 10:00-14:30 IST</t>
-        </is>
-      </c>
-      <c r="G31" s="22" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H31" s="22" t="inlineStr">
-        <is>
-          <t>✅ AGREE</t>
-        </is>
-      </c>
-      <c r="I31" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J31" s="22" t="inlineStr">
-        <is>
-          <t>LargeCap (S&amp;P 500)</t>
-        </is>
-      </c>
-      <c r="K31" s="22" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L31" s="22" t="n"/>
@@ -3564,37 +3552,37 @@
       </c>
       <c r="E32" s="22" t="inlineStr">
         <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F32" s="22" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+      <c r="G32" s="22" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H32" s="22" t="inlineStr">
+        <is>
+          <t>✅ AGREE</t>
+        </is>
+      </c>
+      <c r="I32" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J32" s="22" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="K32" s="22" t="inlineStr">
+        <is>
           <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="F32" s="22" t="inlineStr">
-        <is>
-          <t>🟡 Normal window · 10:00-14:30 IST</t>
-        </is>
-      </c>
-      <c r="G32" s="22" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="H32" s="22" t="inlineStr">
-        <is>
-          <t>✅ AGREE</t>
-        </is>
-      </c>
-      <c r="I32" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J32" s="22" t="inlineStr">
-        <is>
-          <t>LargeCap (S&amp;P 500)</t>
-        </is>
-      </c>
-      <c r="K32" s="22" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
         </is>
       </c>
       <c r="L32" s="22" t="n"/>
@@ -3673,7 +3661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG26"/>
+  <dimension ref="A1:BG38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -9212,6 +9200,2514 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>TRV_USA_20260811</t>
+        </is>
+      </c>
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C27" s="30" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D27" s="30" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="E27" s="30" t="inlineStr">
+        <is>
+          <t>TRV</t>
+        </is>
+      </c>
+      <c r="F27" s="30" t="inlineStr">
+        <is>
+          <t>Travelers</t>
+        </is>
+      </c>
+      <c r="G27" s="30" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H27" s="30" t="n"/>
+      <c r="I27" s="30" t="n"/>
+      <c r="J27" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="K27" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="L27" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="30" t="n">
+        <v>79.3</v>
+      </c>
+      <c r="N27" s="30" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="O27" s="30" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="P27" s="30" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="Q27" s="30" t="inlineStr">
+        <is>
+          <t>FOMC Rate Decision in 1d (high) (+26 more) → -2.0pts · crude +19.8% (rising) → +1.0pts · 12 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
+      <c r="R27" s="30" t="inlineStr">
+        <is>
+          <t>🟢 BUY (Δ-1.0%) · Rank → 1→1 · Conf 57% · band HOLD · 14d left · → BUY</t>
+        </is>
+      </c>
+      <c r="S27" s="30" t="n"/>
+      <c r="T27" s="30" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="U27" s="30" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="V27" s="30" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="W27" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="X27" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y27" s="30" t="n">
+        <v>17</v>
+      </c>
+      <c r="Z27" s="30" t="n">
+        <v>14</v>
+      </c>
+      <c r="AA27" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AB27" s="30" t="n">
+        <v>382.45</v>
+      </c>
+      <c r="AC27" s="30" t="n">
+        <v>382.4500122070312</v>
+      </c>
+      <c r="AD27" s="30" t="n">
+        <v>365.29</v>
+      </c>
+      <c r="AE27" s="30" t="n">
+        <v>372.67</v>
+      </c>
+      <c r="AF27" s="30" t="n">
+        <v>346.84</v>
+      </c>
+      <c r="AG27" s="30" t="n">
+        <v>-9.31</v>
+      </c>
+      <c r="AH27" s="30" t="n">
+        <v>413.26</v>
+      </c>
+      <c r="AI27" s="30" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="AJ27" s="30" t="n">
+        <v>457.54</v>
+      </c>
+      <c r="AK27" s="30" t="n">
+        <v>19.63</v>
+      </c>
+      <c r="AL27" s="30" t="n">
+        <v>382.45</v>
+      </c>
+      <c r="AM27" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN27" s="30" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AO27" s="30" t="n"/>
+      <c r="AP27" s="30" t="n"/>
+      <c r="AQ27" s="30" t="inlineStr">
+        <is>
+          <t>Momentum · Value · Trend</t>
+        </is>
+      </c>
+      <c r="AR27" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AS27" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT27" s="30" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="AU27" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11 04:16</t>
+        </is>
+      </c>
+      <c r="AV27" s="30" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="AW27" s="30" t="inlineStr">
+        <is>
+          <t>🆕 NEW</t>
+        </is>
+      </c>
+      <c r="AX27" s="30" t="n"/>
+      <c r="AY27" s="30" t="inlineStr"/>
+      <c r="AZ27" s="30" t="inlineStr">
+        <is>
+          <t>🟠 PROTECT</t>
+        </is>
+      </c>
+      <c r="BA27" s="30" t="inlineStr">
+        <is>
+          <t>🟡 MEDIUM</t>
+        </is>
+      </c>
+      <c r="BB27" s="30" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BC27" s="30" t="inlineStr">
+        <is>
+          <t>TIGHTEN STOP</t>
+        </is>
+      </c>
+      <c r="BD27" s="30" t="inlineStr">
+        <is>
+          <t>TOMORROW</t>
+        </is>
+      </c>
+      <c r="BE27" s="30" t="inlineStr">
+        <is>
+          <t>Trailing Stop @ 346.84</t>
+        </is>
+      </c>
+      <c r="BF27" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="BG27" s="30" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="31" t="inlineStr">
+        <is>
+          <t>V_USA_20260811</t>
+        </is>
+      </c>
+      <c r="B28" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C28" s="31" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D28" s="31" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="E28" s="31" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F28" s="31" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="G28" s="31" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="H28" s="31" t="n"/>
+      <c r="I28" s="31" t="n"/>
+      <c r="J28" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="K28" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="L28" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="31" t="n">
+        <v>86.5</v>
+      </c>
+      <c r="N28" s="31" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="O28" s="31" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="P28" s="31" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="Q28" s="31" t="inlineStr">
+        <is>
+          <t>FOMC Rate Decision in 1d (high) (+26 more) → -2.0pts · crude +19.8% (rising) → +1.0pts · 5 insider Form 4 filings last 90d → +1.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
+      <c r="R28" s="31" t="inlineStr">
+        <is>
+          <t>🟢 BUY (Δ-3.7%) · Rank → 2→2 · Conf 54% · band STRONG · 14d left · → HOLD</t>
+        </is>
+      </c>
+      <c r="S28" s="31" t="n"/>
+      <c r="T28" s="31" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="U28" s="31" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="V28" s="31" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="W28" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="X28" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="31" t="n">
+        <v>17</v>
+      </c>
+      <c r="Z28" s="31" t="n">
+        <v>14</v>
+      </c>
+      <c r="AA28" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AB28" s="31" t="n">
+        <v>368.54</v>
+      </c>
+      <c r="AC28" s="31" t="n">
+        <v>368.5400085449219</v>
+      </c>
+      <c r="AD28" s="31" t="n">
+        <v>364.85</v>
+      </c>
+      <c r="AE28" s="31" t="n">
+        <v>372.23</v>
+      </c>
+      <c r="AF28" s="31" t="n">
+        <v>350.11</v>
+      </c>
+      <c r="AG28" s="31" t="n">
+        <v>-5</v>
+      </c>
+      <c r="AH28" s="31" t="n">
+        <v>398.02</v>
+      </c>
+      <c r="AI28" s="31" t="n">
+        <v>8</v>
+      </c>
+      <c r="AJ28" s="31" t="n">
+        <v>423.82</v>
+      </c>
+      <c r="AK28" s="31" t="n">
+        <v>15</v>
+      </c>
+      <c r="AL28" s="31" t="n">
+        <v>368.54</v>
+      </c>
+      <c r="AM28" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN28" s="31" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AO28" s="31" t="n"/>
+      <c r="AP28" s="31" t="n"/>
+      <c r="AQ28" s="31" t="inlineStr">
+        <is>
+          <t>Momentum · Trend · Quality</t>
+        </is>
+      </c>
+      <c r="AR28" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AS28" s="31" t="n"/>
+      <c r="AT28" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU28" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11 04:16</t>
+        </is>
+      </c>
+      <c r="AV28" s="31" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="AW28" s="31" t="inlineStr">
+        <is>
+          <t>🆕 NEW</t>
+        </is>
+      </c>
+      <c r="AX28" s="31" t="n"/>
+      <c r="AY28" s="31" t="inlineStr"/>
+      <c r="AZ28" s="31" t="inlineStr">
+        <is>
+          <t>🟠 PROTECT</t>
+        </is>
+      </c>
+      <c r="BA28" s="31" t="inlineStr">
+        <is>
+          <t>🟡 MEDIUM</t>
+        </is>
+      </c>
+      <c r="BB28" s="31" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BC28" s="31" t="inlineStr">
+        <is>
+          <t>TIGHTEN STOP</t>
+        </is>
+      </c>
+      <c r="BD28" s="31" t="inlineStr">
+        <is>
+          <t>TOMORROW</t>
+        </is>
+      </c>
+      <c r="BE28" s="31" t="inlineStr">
+        <is>
+          <t>Trailing Stop @ 350.11</t>
+        </is>
+      </c>
+      <c r="BF28" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="BG28" s="31" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>V_USA_20260811</t>
+        </is>
+      </c>
+      <c r="B29" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D29" s="30" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F29" s="30" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="G29" s="30" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H29" s="30" t="n"/>
+      <c r="I29" s="30" t="n"/>
+      <c r="J29" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" s="30" t="n"/>
+      <c r="L29" s="30" t="n"/>
+      <c r="M29" s="30" t="n">
+        <v>86.5</v>
+      </c>
+      <c r="N29" s="30" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="O29" s="30" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="P29" s="30" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="Q29" s="30" t="inlineStr">
+        <is>
+          <t>FOMC Rate Decision in 1d (high) (+26 more) → -2.0pts · crude +19.8% (rising) → +1.0pts · 5 insider Form 4 filings last 90d → +1.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
+      <c r="R29" s="30" t="inlineStr">
+        <is>
+          <t>🟢 BUY (Δ-2.0%) · Rank #1 · Conf 54% · momentum → · band STRONG · 91d left · → BUY</t>
+        </is>
+      </c>
+      <c r="S29" s="30" t="n"/>
+      <c r="T29" s="30" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="U29" s="30" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="V29" s="30" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="W29" s="30" t="n"/>
+      <c r="X29" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y29" s="30" t="n">
+        <v>90</v>
+      </c>
+      <c r="Z29" s="30" t="n">
+        <v>91</v>
+      </c>
+      <c r="AA29" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AB29" s="30" t="n">
+        <v>368.54</v>
+      </c>
+      <c r="AC29" s="30" t="n">
+        <v>368.5400085449219</v>
+      </c>
+      <c r="AD29" s="30" t="n">
+        <v>351.39</v>
+      </c>
+      <c r="AE29" s="30" t="n">
+        <v>365.73</v>
+      </c>
+      <c r="AF29" s="30" t="n">
+        <v>340.632</v>
+      </c>
+      <c r="AG29" s="30" t="n">
+        <v>-7.57</v>
+      </c>
+      <c r="AH29" s="30" t="n">
+        <v>387.2448000000001</v>
+      </c>
+      <c r="AI29" s="30" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="AJ29" s="30" t="n">
+        <v>414.3519360000001</v>
+      </c>
+      <c r="AK29" s="30" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="AL29" s="30" t="n">
+        <v>368.54</v>
+      </c>
+      <c r="AM29" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN29" s="30" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AO29" s="30" t="n"/>
+      <c r="AP29" s="30" t="n"/>
+      <c r="AQ29" s="30" t="n"/>
+      <c r="AR29" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AS29" s="30" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT29" s="30" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="AU29" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11 04:16</t>
+        </is>
+      </c>
+      <c r="AV29" s="30" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="AW29" s="30" t="inlineStr">
+        <is>
+          <t>🆕 NEW</t>
+        </is>
+      </c>
+      <c r="AX29" s="30" t="n"/>
+      <c r="AY29" s="30" t="inlineStr"/>
+      <c r="AZ29" s="30" t="inlineStr">
+        <is>
+          <t>🟠 PROTECT</t>
+        </is>
+      </c>
+      <c r="BA29" s="30" t="inlineStr">
+        <is>
+          <t>🟡 MEDIUM</t>
+        </is>
+      </c>
+      <c r="BB29" s="30" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BC29" s="30" t="inlineStr">
+        <is>
+          <t>TIGHTEN STOP</t>
+        </is>
+      </c>
+      <c r="BD29" s="30" t="inlineStr">
+        <is>
+          <t>TOMORROW</t>
+        </is>
+      </c>
+      <c r="BE29" s="30" t="inlineStr">
+        <is>
+          <t>Trailing Stop @ 340.63</t>
+        </is>
+      </c>
+      <c r="BF29" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="BG29" s="30" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>TRV_USA_20260811</t>
+        </is>
+      </c>
+      <c r="B30" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C30" s="30" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D30" s="30" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="E30" s="30" t="inlineStr">
+        <is>
+          <t>TRV</t>
+        </is>
+      </c>
+      <c r="F30" s="30" t="inlineStr">
+        <is>
+          <t>Travelers</t>
+        </is>
+      </c>
+      <c r="G30" s="30" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H30" s="30" t="n"/>
+      <c r="I30" s="30" t="n"/>
+      <c r="J30" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="K30" s="30" t="n"/>
+      <c r="L30" s="30" t="n"/>
+      <c r="M30" s="30" t="n">
+        <v>79.3</v>
+      </c>
+      <c r="N30" s="30" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="O30" s="30" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="P30" s="30" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="Q30" s="30" t="inlineStr">
+        <is>
+          <t>FOMC Rate Decision in 1d (high) (+26 more) → -2.0pts · crude +19.8% (rising) → +1.0pts · 12 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
+      <c r="R30" s="30" t="inlineStr">
+        <is>
+          <t>🟢 BUY (Δ-1.0%) · Rank #2 · Conf 57% · momentum → · band HOLD · 91d left · → BUY</t>
+        </is>
+      </c>
+      <c r="S30" s="30" t="n"/>
+      <c r="T30" s="30" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="U30" s="30" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="V30" s="30" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="W30" s="30" t="n"/>
+      <c r="X30" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y30" s="30" t="n">
+        <v>90</v>
+      </c>
+      <c r="Z30" s="30" t="n">
+        <v>91</v>
+      </c>
+      <c r="AA30" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AB30" s="30" t="n">
+        <v>382.45</v>
+      </c>
+      <c r="AC30" s="30" t="n">
+        <v>382.4500122070312</v>
+      </c>
+      <c r="AD30" s="30" t="n">
+        <v>365.29</v>
+      </c>
+      <c r="AE30" s="30" t="n">
+        <v>372.67</v>
+      </c>
+      <c r="AF30" s="30" t="n">
+        <v>350.531</v>
+      </c>
+      <c r="AG30" s="30" t="n">
+        <v>-8.35</v>
+      </c>
+      <c r="AH30" s="30" t="n">
+        <v>413.26</v>
+      </c>
+      <c r="AI30" s="30" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="AJ30" s="30" t="n">
+        <v>442.1882</v>
+      </c>
+      <c r="AK30" s="30" t="n">
+        <v>15.62</v>
+      </c>
+      <c r="AL30" s="30" t="n">
+        <v>382.45</v>
+      </c>
+      <c r="AM30" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN30" s="30" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AO30" s="30" t="n"/>
+      <c r="AP30" s="30" t="n"/>
+      <c r="AQ30" s="30" t="n"/>
+      <c r="AR30" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AS30" s="30" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT30" s="30" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="AU30" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11 04:16</t>
+        </is>
+      </c>
+      <c r="AV30" s="30" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="AW30" s="30" t="inlineStr">
+        <is>
+          <t>🆕 NEW</t>
+        </is>
+      </c>
+      <c r="AX30" s="30" t="n"/>
+      <c r="AY30" s="30" t="inlineStr"/>
+      <c r="AZ30" s="30" t="inlineStr">
+        <is>
+          <t>🟠 PROTECT</t>
+        </is>
+      </c>
+      <c r="BA30" s="30" t="inlineStr">
+        <is>
+          <t>🟡 MEDIUM</t>
+        </is>
+      </c>
+      <c r="BB30" s="30" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BC30" s="30" t="inlineStr">
+        <is>
+          <t>TIGHTEN STOP</t>
+        </is>
+      </c>
+      <c r="BD30" s="30" t="inlineStr">
+        <is>
+          <t>TOMORROW</t>
+        </is>
+      </c>
+      <c r="BE30" s="30" t="inlineStr">
+        <is>
+          <t>Trailing Stop @ 350.53</t>
+        </is>
+      </c>
+      <c r="BF30" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="BG30" s="30" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>NVDA_USA_20260811</t>
+        </is>
+      </c>
+      <c r="B31" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C31" s="30" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D31" s="30" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="E31" s="30" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="F31" s="30" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="G31" s="30" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H31" s="30" t="n"/>
+      <c r="I31" s="30" t="n"/>
+      <c r="J31" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K31" s="30" t="n"/>
+      <c r="L31" s="30" t="n"/>
+      <c r="M31" s="30" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="N31" s="30" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="O31" s="30" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="P31" s="30" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="Q31" s="30" t="inlineStr">
+        <is>
+          <t>FOMC Rate Decision in 1d (high) (+26 more) → -2.0pts · crude +19.8% (rising) → +1.0pts · 21 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
+      <c r="R31" s="30" t="inlineStr">
+        <is>
+          <t>🟢 BUY (Δ-2.0%) · Rank #3 · Conf 47% · momentum → · band HOLD · 91d left · → BUY</t>
+        </is>
+      </c>
+      <c r="S31" s="30" t="inlineStr">
+        <is>
+          <t>WARNING·STOP_LOSS_HIT·-7.5% ≤ -5.0% · exit</t>
+        </is>
+      </c>
+      <c r="T31" s="30" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="U31" s="30" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="V31" s="30" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="W31" s="30" t="n"/>
+      <c r="X31" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y31" s="30" t="n">
+        <v>90</v>
+      </c>
+      <c r="Z31" s="30" t="n">
+        <v>91</v>
+      </c>
+      <c r="AA31" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AB31" s="30" t="n">
+        <v>219.22</v>
+      </c>
+      <c r="AC31" s="30" t="n">
+        <v>219.2200012207031</v>
+      </c>
+      <c r="AD31" s="30" t="n">
+        <v>198.75</v>
+      </c>
+      <c r="AE31" s="30" t="n">
+        <v>206.87</v>
+      </c>
+      <c r="AF31" s="30" t="n">
+        <v>192.6695</v>
+      </c>
+      <c r="AG31" s="30" t="n">
+        <v>-12.11</v>
+      </c>
+      <c r="AH31" s="30" t="n">
+        <v>219.0348</v>
+      </c>
+      <c r="AI31" s="30" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="AJ31" s="30" t="n">
+        <v>234.367236</v>
+      </c>
+      <c r="AK31" s="30" t="n">
+        <v>6.91</v>
+      </c>
+      <c r="AL31" s="30" t="n">
+        <v>219.22</v>
+      </c>
+      <c r="AM31" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN31" s="30" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AO31" s="30" t="n"/>
+      <c r="AP31" s="30" t="n"/>
+      <c r="AQ31" s="30" t="n"/>
+      <c r="AR31" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AS31" s="30" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT31" s="30" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="AU31" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11 04:16</t>
+        </is>
+      </c>
+      <c r="AV31" s="30" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="AW31" s="30" t="inlineStr">
+        <is>
+          <t>🆕 NEW</t>
+        </is>
+      </c>
+      <c r="AX31" s="30" t="n"/>
+      <c r="AY31" s="30" t="inlineStr"/>
+      <c r="AZ31" s="30" t="inlineStr">
+        <is>
+          <t>🟠 PROTECT</t>
+        </is>
+      </c>
+      <c r="BA31" s="30" t="inlineStr">
+        <is>
+          <t>🟡 MEDIUM</t>
+        </is>
+      </c>
+      <c r="BB31" s="30" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BC31" s="30" t="inlineStr">
+        <is>
+          <t>TIGHTEN STOP</t>
+        </is>
+      </c>
+      <c r="BD31" s="30" t="inlineStr">
+        <is>
+          <t>TOMORROW</t>
+        </is>
+      </c>
+      <c r="BE31" s="30" t="inlineStr">
+        <is>
+          <t>Trailing Stop @ 192.67</t>
+        </is>
+      </c>
+      <c r="BF31" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="BG31" s="30" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>MSFT_USA_20260811</t>
+        </is>
+      </c>
+      <c r="B32" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C32" s="30" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D32" s="30" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="E32" s="30" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="F32" s="30" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="G32" s="30" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H32" s="30" t="n"/>
+      <c r="I32" s="30" t="n"/>
+      <c r="J32" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="K32" s="30" t="n"/>
+      <c r="L32" s="30" t="n"/>
+      <c r="M32" s="30" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="N32" s="30" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="O32" s="30" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="P32" s="30" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="Q32" s="30" t="inlineStr">
+        <is>
+          <t>FOMC Rate Decision in 1d (high) (+26 more) → -2.0pts · crude +19.8% (rising) → +1.0pts · 33 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
+      <c r="R32" s="30" t="inlineStr">
+        <is>
+          <t>🟢 BUY (Δ-2.0%) · Rank #4 · Conf 54% · momentum → · band HOLD · 91d left · → BUY</t>
+        </is>
+      </c>
+      <c r="S32" s="30" t="inlineStr">
+        <is>
+          <t>CRITICAL·DEEP_LOSS·-19.2% ≤ -8.0% · EXIT URGENT</t>
+        </is>
+      </c>
+      <c r="T32" s="30" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="U32" s="30" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="V32" s="30" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="W32" s="30" t="n"/>
+      <c r="X32" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y32" s="30" t="n">
+        <v>90</v>
+      </c>
+      <c r="Z32" s="30" t="n">
+        <v>91</v>
+      </c>
+      <c r="AA32" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AB32" s="30" t="n">
+        <v>487.46</v>
+      </c>
+      <c r="AC32" s="30" t="n">
+        <v>487.4599914550781</v>
+      </c>
+      <c r="AD32" s="30" t="n">
+        <v>385.94</v>
+      </c>
+      <c r="AE32" s="30" t="n">
+        <v>401.7</v>
+      </c>
+      <c r="AF32" s="30" t="n">
+        <v>374.129</v>
+      </c>
+      <c r="AG32" s="30" t="n">
+        <v>-23.25</v>
+      </c>
+      <c r="AH32" s="30" t="n">
+        <v>425.3256</v>
+      </c>
+      <c r="AI32" s="30" t="n">
+        <v>-12.75</v>
+      </c>
+      <c r="AJ32" s="30" t="n">
+        <v>455.098392</v>
+      </c>
+      <c r="AK32" s="30" t="n">
+        <v>-6.64</v>
+      </c>
+      <c r="AL32" s="30" t="n">
+        <v>487.46</v>
+      </c>
+      <c r="AM32" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN32" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO32" s="30" t="n"/>
+      <c r="AP32" s="30" t="n"/>
+      <c r="AQ32" s="30" t="n"/>
+      <c r="AR32" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AS32" s="30" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT32" s="30" t="n">
+        <v>-12.75</v>
+      </c>
+      <c r="AU32" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-11 04:16</t>
+        </is>
+      </c>
+      <c r="AV32" s="30" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="AW32" s="30" t="inlineStr">
+        <is>
+          <t>🆕 NEW</t>
+        </is>
+      </c>
+      <c r="AX32" s="30" t="n"/>
+      <c r="AY32" s="30" t="inlineStr"/>
+      <c r="AZ32" s="30" t="inlineStr">
+        <is>
+          <t>🟠 PROTECT</t>
+        </is>
+      </c>
+      <c r="BA32" s="30" t="inlineStr">
+        <is>
+          <t>🟡 MEDIUM</t>
+        </is>
+      </c>
+      <c r="BB32" s="30" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BC32" s="30" t="inlineStr">
+        <is>
+          <t>TIGHTEN STOP</t>
+        </is>
+      </c>
+      <c r="BD32" s="30" t="inlineStr">
+        <is>
+          <t>TOMORROW</t>
+        </is>
+      </c>
+      <c r="BE32" s="30" t="inlineStr">
+        <is>
+          <t>Trailing Stop @ 374.13</t>
+        </is>
+      </c>
+      <c r="BF32" s="30" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="BG32" s="30" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="31" t="inlineStr">
+        <is>
+          <t>KO_USA_20260811</t>
+        </is>
+      </c>
+      <c r="B33" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C33" s="31" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D33" s="31" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="E33" s="31" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="F33" s="31" t="inlineStr">
+        <is>
+          <t>Coca-Cola</t>
+        </is>
+      </c>
+      <c r="G33" s="31" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="H33" s="31" t="n"/>
+      <c r="I33" s="31" t="n"/>
+      <c r="J33" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="K33" s="31" t="n"/>
+      <c r="L33" s="31" t="n"/>
+      <c r="M33" s="31" t="n">
+        <v>84.09999999999999</v>
+      </c>
+      <c r="N33" s="31" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="O33" s="31" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="P33" s="31" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="Q33" s="31" t="inlineStr">
+        <is>
+          <t>FOMC Rate Decision in 1d (high) (+26 more) → -2.0pts · crude +19.8% (rising) → +1.0pts · 11 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
+      <c r="R33" s="31" t="inlineStr">
+        <is>
+          <t>🟢 BUY (Δ-2.0%) · Rank #5 · Conf 50% · momentum → · band STRONG · 91d left · → HOLD</t>
+        </is>
+      </c>
+      <c r="S33" s="31" t="inlineStr">
+        <is>
+          <t>WARNING·STOP_LOSS_HIT·-6.1% ≤ -5.0% · exit</t>
+        </is>
+      </c>
+      <c r="T33" s="31" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="U33" s="31" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="V33" s="31" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="W33" s="31" t="n"/>
+      <c r="X33" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y33" s="31" t="n">
+        <v>90</v>
+      </c>
+      <c r="Z33" s="31" t="n">
+        <v>91</v>
+      </c>
+      <c r="AA33" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AB33" s="31" t="n">
+        <v>86.83</v>
+      </c>
+      <c r="AC33" s="31" t="n">
+        <v>86.83000183105469</v>
+      </c>
+      <c r="AD33" s="31" t="n">
+        <v>79.93000000000001</v>
+      </c>
+      <c r="AE33" s="31" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="AF33" s="31" t="n">
+        <v>77.482</v>
+      </c>
+      <c r="AG33" s="31" t="n">
+        <v>-10.77</v>
+      </c>
+      <c r="AH33" s="31" t="n">
+        <v>88.0848</v>
+      </c>
+      <c r="AI33" s="31" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="AJ33" s="31" t="n">
+        <v>94.250736</v>
+      </c>
+      <c r="AK33" s="31" t="n">
+        <v>8.550000000000001</v>
+      </c>
+      <c r="AL33" s="31" t="n">
+        <v>86.83</v>
+      </c>
+      <c r="AM33" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN33" s="31" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AO33" s="31" t="n"/>
+      <c r="AP33" s="31" t="n"/>
+      <c r="AQ33" s="31" t="n"/>
+      <c r="AR33" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AS33" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT33" s="31" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="AU33" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11 04:16</t>
+        </is>
+      </c>
+      <c r="AV33" s="31" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="AW33" s="31" t="inlineStr">
+        <is>
+          <t>🆕 NEW</t>
+        </is>
+      </c>
+      <c r="AX33" s="31" t="n"/>
+      <c r="AY33" s="31" t="inlineStr"/>
+      <c r="AZ33" s="31" t="inlineStr">
+        <is>
+          <t>🟠 PROTECT</t>
+        </is>
+      </c>
+      <c r="BA33" s="31" t="inlineStr">
+        <is>
+          <t>🟡 MEDIUM</t>
+        </is>
+      </c>
+      <c r="BB33" s="31" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BC33" s="31" t="inlineStr">
+        <is>
+          <t>TIGHTEN STOP</t>
+        </is>
+      </c>
+      <c r="BD33" s="31" t="inlineStr">
+        <is>
+          <t>TOMORROW</t>
+        </is>
+      </c>
+      <c r="BE33" s="31" t="inlineStr">
+        <is>
+          <t>Trailing Stop @ 77.48</t>
+        </is>
+      </c>
+      <c r="BF33" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="BG33" s="31" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="31" t="inlineStr">
+        <is>
+          <t>HON_USA_20260811</t>
+        </is>
+      </c>
+      <c r="B34" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C34" s="31" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D34" s="31" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="E34" s="31" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
+      <c r="F34" s="31" t="inlineStr">
+        <is>
+          <t>Honeywell</t>
+        </is>
+      </c>
+      <c r="G34" s="31" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="H34" s="31" t="n"/>
+      <c r="I34" s="31" t="n"/>
+      <c r="J34" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="K34" s="31" t="n"/>
+      <c r="L34" s="31" t="n"/>
+      <c r="M34" s="31" t="n">
+        <v>76</v>
+      </c>
+      <c r="N34" s="31" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="O34" s="31" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="P34" s="31" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="Q34" s="31" t="inlineStr">
+        <is>
+          <t>FOMC Rate Decision in 1d (high) (+26 more) → -2.0pts · crude +19.8% (rising) → +1.0pts · 48 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
+      <c r="R34" s="31" t="inlineStr">
+        <is>
+          <t>🟢 BUY (Δ-2.0%) · Rank #6 · Conf 50% · momentum → · band HOLD · 91d left · → HOLD</t>
+        </is>
+      </c>
+      <c r="S34" s="31" t="inlineStr">
+        <is>
+          <t>CRITICAL·DEEP_LOSS·-9.3% ≤ -8.0% · EXIT URGENT</t>
+        </is>
+      </c>
+      <c r="T34" s="31" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="U34" s="31" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="V34" s="31" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="W34" s="31" t="n"/>
+      <c r="X34" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y34" s="31" t="n">
+        <v>90</v>
+      </c>
+      <c r="Z34" s="31" t="n">
+        <v>91</v>
+      </c>
+      <c r="AA34" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AB34" s="31" t="n">
+        <v>248.12</v>
+      </c>
+      <c r="AC34" s="31" t="n">
+        <v>248.1199951171875</v>
+      </c>
+      <c r="AD34" s="31" t="n">
+        <v>220.52</v>
+      </c>
+      <c r="AE34" s="31" t="n">
+        <v>229.52</v>
+      </c>
+      <c r="AF34" s="31" t="n">
+        <v>213.769</v>
+      </c>
+      <c r="AG34" s="31" t="n">
+        <v>-13.84</v>
+      </c>
+      <c r="AH34" s="31" t="n">
+        <v>243.0216</v>
+      </c>
+      <c r="AI34" s="31" t="n">
+        <v>-2.05</v>
+      </c>
+      <c r="AJ34" s="31" t="n">
+        <v>260.0331120000001</v>
+      </c>
+      <c r="AK34" s="31" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="AL34" s="31" t="n">
+        <v>248.12</v>
+      </c>
+      <c r="AM34" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN34" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO34" s="31" t="n"/>
+      <c r="AP34" s="31" t="n"/>
+      <c r="AQ34" s="31" t="n"/>
+      <c r="AR34" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AS34" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT34" s="31" t="n">
+        <v>-2.05</v>
+      </c>
+      <c r="AU34" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11 04:16</t>
+        </is>
+      </c>
+      <c r="AV34" s="31" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="AW34" s="31" t="inlineStr">
+        <is>
+          <t>🆕 NEW</t>
+        </is>
+      </c>
+      <c r="AX34" s="31" t="n"/>
+      <c r="AY34" s="31" t="inlineStr"/>
+      <c r="AZ34" s="31" t="inlineStr">
+        <is>
+          <t>🟠 PROTECT</t>
+        </is>
+      </c>
+      <c r="BA34" s="31" t="inlineStr">
+        <is>
+          <t>🟡 MEDIUM</t>
+        </is>
+      </c>
+      <c r="BB34" s="31" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BC34" s="31" t="inlineStr">
+        <is>
+          <t>TIGHTEN STOP</t>
+        </is>
+      </c>
+      <c r="BD34" s="31" t="inlineStr">
+        <is>
+          <t>TOMORROW</t>
+        </is>
+      </c>
+      <c r="BE34" s="31" t="inlineStr">
+        <is>
+          <t>Trailing Stop @ 213.77</t>
+        </is>
+      </c>
+      <c r="BF34" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="BG34" s="31" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="31" t="inlineStr">
+        <is>
+          <t>AAPL_USA_20260811</t>
+        </is>
+      </c>
+      <c r="B35" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C35" s="31" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D35" s="31" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="E35" s="31" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="F35" s="31" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="G35" s="31" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="H35" s="31" t="n"/>
+      <c r="I35" s="31" t="n"/>
+      <c r="J35" s="31" t="n">
+        <v>7</v>
+      </c>
+      <c r="K35" s="31" t="n"/>
+      <c r="L35" s="31" t="n"/>
+      <c r="M35" s="31" t="n">
+        <v>83.5</v>
+      </c>
+      <c r="N35" s="31" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="O35" s="31" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="P35" s="31" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="Q35" s="31" t="inlineStr">
+        <is>
+          <t>FOMC Rate Decision in 1d (high) (+26 more) → -2.0pts · crude +19.8% (rising) → +1.0pts · 5 insider Form 4 filings last 90d → +1.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
+      <c r="R35" s="31" t="inlineStr">
+        <is>
+          <t>🟢 BUY (Δ-2.0%) · Rank #7 · Conf 50% · momentum → · band STRONG · 91d left · → HOLD</t>
+        </is>
+      </c>
+      <c r="S35" s="31" t="n"/>
+      <c r="T35" s="31" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="U35" s="31" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="V35" s="31" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="W35" s="31" t="n"/>
+      <c r="X35" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y35" s="31" t="n">
+        <v>90</v>
+      </c>
+      <c r="Z35" s="31" t="n">
+        <v>91</v>
+      </c>
+      <c r="AA35" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AB35" s="31" t="n">
+        <v>311</v>
+      </c>
+      <c r="AC35" s="31" t="n">
+        <v>311</v>
+      </c>
+      <c r="AD35" s="31" t="n">
+        <v>327.07</v>
+      </c>
+      <c r="AE35" s="31" t="n">
+        <v>340.41</v>
+      </c>
+      <c r="AF35" s="31" t="n">
+        <v>317.053</v>
+      </c>
+      <c r="AG35" s="31" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="AH35" s="31" t="n">
+        <v>360.4392</v>
+      </c>
+      <c r="AI35" s="31" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="AJ35" s="31" t="n">
+        <v>385.669944</v>
+      </c>
+      <c r="AK35" s="31" t="n">
+        <v>24.01</v>
+      </c>
+      <c r="AL35" s="31" t="n">
+        <v>311</v>
+      </c>
+      <c r="AM35" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN35" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO35" s="31" t="n"/>
+      <c r="AP35" s="31" t="n"/>
+      <c r="AQ35" s="31" t="n"/>
+      <c r="AR35" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AS35" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT35" s="31" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="AU35" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11 04:16</t>
+        </is>
+      </c>
+      <c r="AV35" s="31" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="AW35" s="31" t="inlineStr">
+        <is>
+          <t>🆕 NEW</t>
+        </is>
+      </c>
+      <c r="AX35" s="31" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="AY35" s="31" t="inlineStr">
+        <is>
+          <t>🏆 QUALITY</t>
+        </is>
+      </c>
+      <c r="AZ35" s="31" t="inlineStr">
+        <is>
+          <t>🟢 HOLD</t>
+        </is>
+      </c>
+      <c r="BA35" s="31" t="inlineStr">
+        <is>
+          <t>🟢 LOW</t>
+        </is>
+      </c>
+      <c r="BB35" s="31" t="inlineStr">
+        <is>
+          <t>Compounder</t>
+        </is>
+      </c>
+      <c r="BC35" s="31" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="BD35" s="31" t="inlineStr">
+        <is>
+          <t>30 DAYS</t>
+        </is>
+      </c>
+      <c r="BE35" s="31" t="inlineStr">
+        <is>
+          <t>Watching @ 360.44</t>
+        </is>
+      </c>
+      <c r="BF35" s="31" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="BG35" s="31" t="inlineStr">
+        <is>
+          <t>⚪ No immediate execution</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="31" t="inlineStr">
+        <is>
+          <t>JPM_USA_20260811</t>
+        </is>
+      </c>
+      <c r="B36" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C36" s="31" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D36" s="31" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="E36" s="31" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="F36" s="31" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase</t>
+        </is>
+      </c>
+      <c r="G36" s="31" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="H36" s="31" t="n"/>
+      <c r="I36" s="31" t="n"/>
+      <c r="J36" s="31" t="n">
+        <v>8</v>
+      </c>
+      <c r="K36" s="31" t="n"/>
+      <c r="L36" s="31" t="n"/>
+      <c r="M36" s="31" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="N36" s="31" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="O36" s="31" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="P36" s="31" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="Q36" s="31" t="inlineStr">
+        <is>
+          <t>FOMC Rate Decision in 1d (high) (+26 more) → -2.0pts · crude +19.8% (rising) → +1.0pts · 18 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
+      <c r="R36" s="31" t="inlineStr">
+        <is>
+          <t>🟢 BUY (Δ-2.0%) · Rank #8 · Conf 50% · momentum → · band HOLD · 91d left · → HOLD</t>
+        </is>
+      </c>
+      <c r="S36" s="31" t="inlineStr">
+        <is>
+          <t>WARNING·STOP_LOSS_HIT·-5.0% ≤ -5.0% · exit</t>
+        </is>
+      </c>
+      <c r="T36" s="31" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="U36" s="31" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="V36" s="31" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="W36" s="31" t="n"/>
+      <c r="X36" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y36" s="31" t="n">
+        <v>90</v>
+      </c>
+      <c r="Z36" s="31" t="n">
+        <v>91</v>
+      </c>
+      <c r="AA36" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AB36" s="31" t="n">
+        <v>359.24</v>
+      </c>
+      <c r="AC36" s="31" t="n">
+        <v>359.239990234375</v>
+      </c>
+      <c r="AD36" s="31" t="n">
+        <v>334.28</v>
+      </c>
+      <c r="AE36" s="31" t="n">
+        <v>347.92</v>
+      </c>
+      <c r="AF36" s="31" t="n">
+        <v>324.045</v>
+      </c>
+      <c r="AG36" s="31" t="n">
+        <v>-9.800000000000001</v>
+      </c>
+      <c r="AH36" s="31" t="n">
+        <v>368.388</v>
+      </c>
+      <c r="AI36" s="31" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="AJ36" s="31" t="n">
+        <v>394.1751600000001</v>
+      </c>
+      <c r="AK36" s="31" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="AL36" s="31" t="n">
+        <v>359.24</v>
+      </c>
+      <c r="AM36" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN36" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO36" s="31" t="n"/>
+      <c r="AP36" s="31" t="n"/>
+      <c r="AQ36" s="31" t="n"/>
+      <c r="AR36" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AS36" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT36" s="31" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="AU36" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11 04:16</t>
+        </is>
+      </c>
+      <c r="AV36" s="31" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="AW36" s="31" t="inlineStr">
+        <is>
+          <t>🆕 NEW</t>
+        </is>
+      </c>
+      <c r="AX36" s="31" t="n"/>
+      <c r="AY36" s="31" t="inlineStr"/>
+      <c r="AZ36" s="31" t="inlineStr">
+        <is>
+          <t>🟠 PROTECT</t>
+        </is>
+      </c>
+      <c r="BA36" s="31" t="inlineStr">
+        <is>
+          <t>🟡 MEDIUM</t>
+        </is>
+      </c>
+      <c r="BB36" s="31" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BC36" s="31" t="inlineStr">
+        <is>
+          <t>TIGHTEN STOP</t>
+        </is>
+      </c>
+      <c r="BD36" s="31" t="inlineStr">
+        <is>
+          <t>TOMORROW</t>
+        </is>
+      </c>
+      <c r="BE36" s="31" t="inlineStr">
+        <is>
+          <t>Trailing Stop @ 324.05</t>
+        </is>
+      </c>
+      <c r="BF36" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="BG36" s="31" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="31" t="inlineStr">
+        <is>
+          <t>GS_USA_20260811</t>
+        </is>
+      </c>
+      <c r="B37" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C37" s="31" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D37" s="31" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="E37" s="31" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="F37" s="31" t="inlineStr">
+        <is>
+          <t>Goldman Sachs</t>
+        </is>
+      </c>
+      <c r="G37" s="31" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="H37" s="31" t="n"/>
+      <c r="I37" s="31" t="n"/>
+      <c r="J37" s="31" t="n">
+        <v>9</v>
+      </c>
+      <c r="K37" s="31" t="n"/>
+      <c r="L37" s="31" t="n"/>
+      <c r="M37" s="31" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="N37" s="31" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="O37" s="31" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="P37" s="31" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="Q37" s="31" t="inlineStr">
+        <is>
+          <t>FOMC Rate Decision in 1d (high) (+26 more) → -2.0pts · crude +19.8% (rising) → +1.0pts · 9 insider Form 4 filings last 90d → +1.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
+      <c r="R37" s="31" t="inlineStr">
+        <is>
+          <t>🟢 BUY (Δ-2.0%) · Rank #9 · Conf 51% · momentum → · band HOLD · 91d left · → HOLD</t>
+        </is>
+      </c>
+      <c r="S37" s="31" t="n"/>
+      <c r="T37" s="31" t="n">
+        <v>51</v>
+      </c>
+      <c r="U37" s="31" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="V37" s="31" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="W37" s="31" t="n"/>
+      <c r="X37" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y37" s="31" t="n">
+        <v>90</v>
+      </c>
+      <c r="Z37" s="31" t="n">
+        <v>91</v>
+      </c>
+      <c r="AA37" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AB37" s="31" t="n">
+        <v>1060.38</v>
+      </c>
+      <c r="AC37" s="31" t="n">
+        <v>1060.380004882812</v>
+      </c>
+      <c r="AD37" s="31" t="n">
+        <v>1043.92</v>
+      </c>
+      <c r="AE37" s="31" t="n">
+        <v>1086.52</v>
+      </c>
+      <c r="AF37" s="31" t="n">
+        <v>1011.959</v>
+      </c>
+      <c r="AG37" s="31" t="n">
+        <v>-4.57</v>
+      </c>
+      <c r="AH37" s="31" t="n">
+        <v>1150.4376</v>
+      </c>
+      <c r="AI37" s="31" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="AJ37" s="31" t="n">
+        <v>1230.968232</v>
+      </c>
+      <c r="AK37" s="31" t="n">
+        <v>16.09</v>
+      </c>
+      <c r="AL37" s="31" t="n">
+        <v>1060.38</v>
+      </c>
+      <c r="AM37" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN37" s="31" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AO37" s="31" t="n"/>
+      <c r="AP37" s="31" t="n"/>
+      <c r="AQ37" s="31" t="n"/>
+      <c r="AR37" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AS37" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT37" s="31" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="AU37" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11 04:16</t>
+        </is>
+      </c>
+      <c r="AV37" s="31" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="AW37" s="31" t="inlineStr">
+        <is>
+          <t>🆕 NEW</t>
+        </is>
+      </c>
+      <c r="AX37" s="31" t="n"/>
+      <c r="AY37" s="31" t="inlineStr"/>
+      <c r="AZ37" s="31" t="inlineStr">
+        <is>
+          <t>🟠 PROTECT</t>
+        </is>
+      </c>
+      <c r="BA37" s="31" t="inlineStr">
+        <is>
+          <t>🟡 MEDIUM</t>
+        </is>
+      </c>
+      <c r="BB37" s="31" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BC37" s="31" t="inlineStr">
+        <is>
+          <t>TIGHTEN STOP</t>
+        </is>
+      </c>
+      <c r="BD37" s="31" t="inlineStr">
+        <is>
+          <t>TOMORROW</t>
+        </is>
+      </c>
+      <c r="BE37" s="31" t="inlineStr">
+        <is>
+          <t>Trailing Stop @ 1011.96</t>
+        </is>
+      </c>
+      <c r="BF37" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="BG37" s="31" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="31" t="inlineStr">
+        <is>
+          <t>MMM_USA_20260811</t>
+        </is>
+      </c>
+      <c r="B38" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C38" s="31" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D38" s="31" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="E38" s="31" t="inlineStr">
+        <is>
+          <t>MMM</t>
+        </is>
+      </c>
+      <c r="F38" s="31" t="inlineStr">
+        <is>
+          <t>3M</t>
+        </is>
+      </c>
+      <c r="G38" s="31" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="H38" s="31" t="n"/>
+      <c r="I38" s="31" t="n"/>
+      <c r="J38" s="31" t="n">
+        <v>10</v>
+      </c>
+      <c r="K38" s="31" t="n"/>
+      <c r="L38" s="31" t="n"/>
+      <c r="M38" s="31" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="N38" s="31" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="O38" s="31" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="P38" s="31" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="Q38" s="31" t="inlineStr">
+        <is>
+          <t>FOMC Rate Decision in 1d (high) (+26 more) → -2.0pts · crude +19.8% (rising) → +1.0pts · 15 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
+      <c r="R38" s="31" t="inlineStr">
+        <is>
+          <t>🟢 BUY (Δ-2.0%) · Rank #10 · Conf 54% · momentum → · band HOLD · 91d left · → HOLD</t>
+        </is>
+      </c>
+      <c r="S38" s="31" t="inlineStr">
+        <is>
+          <t>CRITICAL·DEEP_LOSS·-12.2% ≤ -8.0% · EXIT URGENT</t>
+        </is>
+      </c>
+      <c r="T38" s="31" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="U38" s="31" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="V38" s="31" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="W38" s="31" t="n"/>
+      <c r="X38" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y38" s="31" t="n">
+        <v>90</v>
+      </c>
+      <c r="Z38" s="31" t="n">
+        <v>91</v>
+      </c>
+      <c r="AA38" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AB38" s="31" t="n">
+        <v>182.08</v>
+      </c>
+      <c r="AC38" s="31" t="n">
+        <v>182.0800018310547</v>
+      </c>
+      <c r="AD38" s="31" t="n">
+        <v>156.64</v>
+      </c>
+      <c r="AE38" s="31" t="n">
+        <v>163.04</v>
+      </c>
+      <c r="AF38" s="31" t="n">
+        <v>151.848</v>
+      </c>
+      <c r="AG38" s="31" t="n">
+        <v>-16.6</v>
+      </c>
+      <c r="AH38" s="31" t="n">
+        <v>172.6272</v>
+      </c>
+      <c r="AI38" s="31" t="n">
+        <v>-5.19</v>
+      </c>
+      <c r="AJ38" s="31" t="n">
+        <v>184.711104</v>
+      </c>
+      <c r="AK38" s="31" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="AL38" s="31" t="n">
+        <v>182.08</v>
+      </c>
+      <c r="AM38" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN38" s="31" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AO38" s="31" t="n"/>
+      <c r="AP38" s="31" t="n"/>
+      <c r="AQ38" s="31" t="n"/>
+      <c r="AR38" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AS38" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT38" s="31" t="n">
+        <v>-5.19</v>
+      </c>
+      <c r="AU38" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-11 04:16</t>
+        </is>
+      </c>
+      <c r="AV38" s="31" t="inlineStr">
+        <is>
+          <t>LargeCap (S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="AW38" s="31" t="inlineStr">
+        <is>
+          <t>🆕 NEW</t>
+        </is>
+      </c>
+      <c r="AX38" s="31" t="n"/>
+      <c r="AY38" s="31" t="inlineStr"/>
+      <c r="AZ38" s="31" t="inlineStr">
+        <is>
+          <t>🟠 PROTECT</t>
+        </is>
+      </c>
+      <c r="BA38" s="31" t="inlineStr">
+        <is>
+          <t>🟡 MEDIUM</t>
+        </is>
+      </c>
+      <c r="BB38" s="31" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BC38" s="31" t="inlineStr">
+        <is>
+          <t>TIGHTEN STOP</t>
+        </is>
+      </c>
+      <c r="BD38" s="31" t="inlineStr">
+        <is>
+          <t>TOMORROW</t>
+        </is>
+      </c>
+      <c r="BE38" s="31" t="inlineStr">
+        <is>
+          <t>Trailing Stop @ 151.85</t>
+        </is>
+      </c>
+      <c r="BF38" s="31" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="BG38" s="31" t="inlineStr">
+        <is>
+          <t>🟡 Normal window · 10:00-14:30 IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>